<commit_message>
Resolve merge conflict for tree_book.html
</commit_message>
<xml_diff>
--- a/data/book_record.xlsx
+++ b/data/book_record.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="521">
   <si>
     <t>title</t>
   </si>
@@ -1568,6 +1568,12 @@
   </si>
   <si>
     <t>Richard Matheson</t>
+  </si>
+  <si>
+    <t>Artemis</t>
+  </si>
+  <si>
+    <t>Andy Weir</t>
   </si>
 </sst>
 </file>
@@ -2778,7 +2784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J222"/>
+  <dimension ref="A1:J223"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="47.9688" style="1" customWidth="1"/>
@@ -9539,6 +9545,36 @@
         <v>2026</v>
       </c>
     </row>
+    <row r="223" ht="13.55" customHeight="1">
+      <c r="A223" t="s" s="5">
+        <v>519</v>
+      </c>
+      <c r="B223" t="s" s="5">
+        <v>520</v>
+      </c>
+      <c r="C223" t="s" s="5">
+        <v>25</v>
+      </c>
+      <c r="D223" t="s" s="5">
+        <v>71</v>
+      </c>
+      <c r="E223" t="s" s="5">
+        <v>14</v>
+      </c>
+      <c r="F223" t="s" s="5">
+        <v>48</v>
+      </c>
+      <c r="G223" t="s" s="5">
+        <v>16</v>
+      </c>
+      <c r="H223" t="s" s="5">
+        <v>415</v>
+      </c>
+      <c r="I223" s="7"/>
+      <c r="J223" s="6">
+        <v>2026</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>